<commit_message>
feat: Implement Visa transaction description cleanup to enhance readability by removing reference numbers
</commit_message>
<xml_diff>
--- a/temp/BBVA_VISA_20250130.xlsx
+++ b/temp/BBVA_VISA_20250130.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>071512K MERPAGO*THOMAS</t>
+          <t>MERPAGO*THOMAS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -517,7 +517,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>000988* ELECTROPAGO*REC PIZZA SA</t>
+          <t>ELECTROPAGO*REC PIZZA SA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>891733K MERPAGO*LUCKY13</t>
+          <t>MERPAGO*LUCKY13</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -571,7 +571,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>504070* TOMATE</t>
+          <t>TOMATE</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>000175K AXION BONPLAND</t>
+          <t>AXION BONPLAND</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>002157* SANDRULI SRL</t>
+          <t>SANDRULI SRL</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -652,7 +652,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>093709Q NETFLIX.COM 42785628363430465</t>
+          <t>NETFLIX.COM 42785628363430465</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>000001* AUTOPISTAS URBAN 000000003616132</t>
+          <t>AUTOPISTAS URBAN 000000003616132</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -706,7 +706,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>152724K MERPAGO*FARMACITY</t>
+          <t>MERPAGO*FARMACITY</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -733,7 +733,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>062195K MERPAGO*THOMAS</t>
+          <t>MERPAGO*THOMAS</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -760,7 +760,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>537338K MERPAGO*QR</t>
+          <t>MERPAGO*QR</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>157805K MERPAGO*FARMACITY</t>
+          <t>MERPAGO*FARMACITY</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -814,7 +814,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>412396K MERPAGO*VEAEXPRESS</t>
+          <t>MERPAGO*VEAEXPRESS</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>000877K AXION BONPLAND</t>
+          <t>AXION BONPLAND</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>994537* BBVA SEGUROS A2052000420510-023-000</t>
+          <t>BBVA SEGUROS A2052000420510-023-000</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -895,7 +895,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>990897* Melé</t>
+          <t>Melé</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>022849K PEDIDOSYA RESTAURANTE</t>
+          <t>PEDIDOSYA RESTAURANTE</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>011651* TRIUNFO COOP D0000007681097-094-004</t>
+          <t>TRIUNFO COOP D0000007681097-094-004</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -976,7 +976,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>112297K PEDIDOSYA PROPINAS</t>
+          <t>PEDIDOSYA PROPINAS</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>006603* RAPPI</t>
+          <t>RAPPI</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>362503V Spotify</t>
+          <t>Spotify</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>990015K MERPAGO*QR</t>
+          <t>MERPAGO*QR</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>987147K MERPAGO*KOPI</t>
+          <t>MERPAGO*KOPI</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>521578K MERPAGO*QR</t>
+          <t>MERPAGO*QR</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>873678K MERPAGO*METROGASSA</t>
+          <t>MERPAGO*METROGASSA</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1165,7 +1165,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>279419K MERPAGO*THOMAS</t>
+          <t>MERPAGO*THOMAS</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>218966K MERPAGO*THOMAS</t>
+          <t>MERPAGO*THOMAS</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>292402K MERPAGO*FARMACITY</t>
+          <t>MERPAGO*FARMACITY</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>135742* PATENTES</t>
+          <t>PATENTES</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>003474* EDENORDIGITAL</t>
+          <t>EDENORDIGITAL</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1300,7 +1300,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>002130K RINCON NORTENO COLEGIALES</t>
+          <t>RINCON NORTENO COLEGIALES</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>158049K MERPAGO*LUCKY13</t>
+          <t>MERPAGO*LUCKY13</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>002547K AXION BONPLAND</t>
+          <t>AXION BONPLAND</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>943671K MERPAGO*TELEPASE</t>
+          <t>MERPAGO*TELEPASE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>120415* EXPERTA SEGURO0000032131884-015-004</t>
+          <t>EXPERTA SEGURO0000032131884-015-004</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>003593* DLO*RAPPI</t>
+          <t>DLO*RAPPI</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1462,7 +1462,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>003289* SANDRULI SRL</t>
+          <t>SANDRULI SRL</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">

</xml_diff>